<commit_message>
refactor: simplify excel reading logic and add automatic CPF padding for leading zeros
</commit_message>
<xml_diff>
--- a/upload/EXCEL/modelo_importacao_vr.xlsx
+++ b/upload/EXCEL/modelo_importacao_vr.xlsx
@@ -21,12 +21,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="225">
-  <si>
-    <t xml:space="preserve">cnpj_condominio*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_condominio*</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="497" uniqueCount="218">
+  <si>
+    <t xml:space="preserve">cnpj_condominio</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_condominio</t>
   </si>
   <si>
     <t xml:space="preserve">tipo_local_condominio</t>
@@ -53,13 +53,13 @@
     <t xml:space="preserve">cep_condominio</t>
   </si>
   <si>
-    <t xml:space="preserve">cpf_funcionario*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">matricula_funcionario*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nome_funcionario*</t>
+    <t xml:space="preserve">cpf_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">matricula_funcionario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_funcionario</t>
   </si>
   <si>
     <t xml:space="preserve">funcao_funcionario</t>
@@ -92,10 +92,10 @@
     <t xml:space="preserve">nome_produto</t>
   </si>
   <si>
-    <t xml:space="preserve">data_competencia*</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valor_beneficio(total)*</t>
+    <t xml:space="preserve">data_competencia</t>
+  </si>
+  <si>
+    <t xml:space="preserve">valor_beneficio(total)</t>
   </si>
   <si>
     <t xml:space="preserve">quantidade_dias</t>
@@ -455,9 +455,6 @@
     <t xml:space="preserve">A</t>
   </si>
   <si>
-    <t xml:space="preserve">cnpj_condominio</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sim *</t>
   </si>
   <si>
@@ -467,9 +464,6 @@
     <t xml:space="preserve">B</t>
   </si>
   <si>
-    <t xml:space="preserve">nome_condominio</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nome/Razão social do condomínio</t>
   </si>
   <si>
@@ -527,27 +521,18 @@
     <t xml:space="preserve">K</t>
   </si>
   <si>
-    <t xml:space="preserve">cpf_funcionario</t>
-  </si>
-  <si>
     <t xml:space="preserve">CPF do funcionário (apenas números, 11 dígitos)</t>
   </si>
   <si>
     <t xml:space="preserve">L</t>
   </si>
   <si>
-    <t xml:space="preserve">matricula_funcionario</t>
-  </si>
-  <si>
     <t xml:space="preserve">Matrícula do funcionário</t>
   </si>
   <si>
     <t xml:space="preserve">M</t>
   </si>
   <si>
-    <t xml:space="preserve">nome_funcionario</t>
-  </si>
-  <si>
     <t xml:space="preserve">Nome completo do funcionário</t>
   </si>
   <si>
@@ -614,16 +599,10 @@
     <t xml:space="preserve">X</t>
   </si>
   <si>
-    <t xml:space="preserve">data_competencia</t>
-  </si>
-  <si>
     <t xml:space="preserve">Data de competência (dd/mm/aaaa)</t>
   </si>
   <si>
     <t xml:space="preserve">Y</t>
-  </si>
-  <si>
-    <t xml:space="preserve">valor_beneficio(total)</t>
   </si>
   <si>
     <t xml:space="preserve">Valor total do benefício em R$</t>
@@ -1002,62 +981,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="21">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F4E78"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF000000"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFF8D7DA"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFC7CE"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF9C0006"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="14">
     <dxf>
       <font>
         <name val="Calibri"/>
@@ -1502,7 +1426,7 @@
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="14.25" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52.49"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="52.48"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="24.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="28.98"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="22.44"/>
@@ -1515,7 +1439,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="2" width="24.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="1" width="37.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="1" width="21.04"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="3" width="29.96"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="3" width="29.97"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="1" width="19.24"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="1" width="18.26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="1" width="27.17"/>
@@ -1662,7 +1586,9 @@
       <c r="X2" s="3" t="n">
         <v>46204</v>
       </c>
-      <c r="Y2" s="13"/>
+      <c r="Y2" s="13" t="n">
+        <v>136</v>
+      </c>
       <c r="Z2" s="1" t="n">
         <v>22</v>
       </c>
@@ -1719,7 +1645,9 @@
       <c r="X3" s="3" t="n">
         <v>46204</v>
       </c>
-      <c r="Y3" s="13"/>
+      <c r="Y3" s="13" t="n">
+        <v>136</v>
+      </c>
       <c r="Z3" s="1" t="n">
         <v>22</v>
       </c>
@@ -1776,7 +1704,9 @@
       <c r="X4" s="3" t="n">
         <v>46204</v>
       </c>
-      <c r="Y4" s="13"/>
+      <c r="Y4" s="13" t="n">
+        <v>136</v>
+      </c>
       <c r="Z4" s="1" t="n">
         <v>22</v>
       </c>
@@ -3084,46 +3014,46 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <conditionalFormatting sqref="B2:B20 D2:D20 G2:J20 M2:M12 M14:M20">
-    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="vencer" dxfId="7">
+    <cfRule type="containsText" priority="2" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="vencer" dxfId="0">
       <formula>NOT(ISERROR(SEARCH("vencer",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Vencido" dxfId="8">
+    <cfRule type="containsText" priority="3" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Vencido" dxfId="1">
       <formula>NOT(ISERROR(SEARCH("Vencido",B2)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="4" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Válido" dxfId="9">
+    <cfRule type="containsText" priority="4" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Válido" dxfId="2">
       <formula>NOT(ISERROR(SEARCH("Válido",B2)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K22:L23 K25:L25">
-    <cfRule type="duplicateValues" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="10"/>
-    <cfRule type="duplicateValues" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11"/>
-    <cfRule type="duplicateValues" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="12"/>
+    <cfRule type="duplicateValues" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3"/>
+    <cfRule type="duplicateValues" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4"/>
+    <cfRule type="duplicateValues" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K25:L25">
-    <cfRule type="duplicateValues" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="13"/>
+    <cfRule type="duplicateValues" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K22:L23">
-    <cfRule type="duplicateValues" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14"/>
+    <cfRule type="duplicateValues" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="M14">
-    <cfRule type="containsText" priority="10" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="vencer" dxfId="15">
+    <cfRule type="containsText" priority="10" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="vencer" dxfId="8">
       <formula>NOT(ISERROR(SEARCH("vencer",M14)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="11" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Vencido" dxfId="16">
+    <cfRule type="containsText" priority="11" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Vencido" dxfId="9">
       <formula>NOT(ISERROR(SEARCH("Vencido",M14)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="12" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Válido" dxfId="17">
+    <cfRule type="containsText" priority="12" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Válido" dxfId="10">
       <formula>NOT(ISERROR(SEARCH("Válido",M14)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M14:M25">
-    <cfRule type="containsText" priority="13" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="vencer" dxfId="18">
+    <cfRule type="containsText" priority="13" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="vencer" dxfId="11">
       <formula>NOT(ISERROR(SEARCH("vencer",M14)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="14" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Vencido" dxfId="19">
+    <cfRule type="containsText" priority="14" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Vencido" dxfId="12">
       <formula>NOT(ISERROR(SEARCH("Vencido",M14)))</formula>
     </cfRule>
-    <cfRule type="containsText" priority="15" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Válido" dxfId="20">
+    <cfRule type="containsText" priority="15" operator="containsText" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="Válido" dxfId="13">
       <formula>NOT(ISERROR(SEARCH("Válido",M14)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3234,462 +3164,462 @@
         <v>143</v>
       </c>
       <c r="B17" s="21" t="s">
+        <v>0</v>
+      </c>
+      <c r="C17" s="21" t="s">
         <v>144</v>
       </c>
-      <c r="C17" s="21" t="s">
+      <c r="D17" s="21" t="s">
         <v>145</v>
-      </c>
-      <c r="D17" s="21" t="s">
-        <v>146</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="21" t="s">
+        <v>146</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>144</v>
+      </c>
+      <c r="D18" s="21" t="s">
         <v>147</v>
-      </c>
-      <c r="B18" s="21" t="s">
-        <v>148</v>
-      </c>
-      <c r="C18" s="21" t="s">
-        <v>145</v>
-      </c>
-      <c r="D18" s="21" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="22" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B19" s="22" t="s">
         <v>2</v>
       </c>
       <c r="C19" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="21" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B20" s="21" t="s">
         <v>3</v>
       </c>
       <c r="C20" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D20" s="21" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="21" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B21" s="21" t="s">
         <v>4</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D21" s="21" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="22" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="B22" s="22" t="s">
         <v>5</v>
       </c>
       <c r="C22" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D22" s="22" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="21" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B23" s="21" t="s">
         <v>6</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="21" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B24" s="21" t="s">
         <v>7</v>
       </c>
       <c r="C24" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D24" s="21" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="21" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="B25" s="21" t="s">
         <v>8</v>
       </c>
       <c r="C25" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D25" s="21" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="21" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B26" s="21" t="s">
         <v>9</v>
       </c>
       <c r="C26" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D26" s="21" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="21" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B27" s="21" t="s">
-        <v>168</v>
+        <v>10</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D27" s="21" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="21" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="B28" s="21" t="s">
-        <v>171</v>
+        <v>11</v>
       </c>
       <c r="C28" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D28" s="21" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B29" s="21" t="s">
-        <v>174</v>
+        <v>12</v>
       </c>
       <c r="C29" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D29" s="21" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="22" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="B30" s="22" t="s">
         <v>13</v>
       </c>
       <c r="C30" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D30" s="22" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="21" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="B31" s="21" t="s">
         <v>14</v>
       </c>
       <c r="C31" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D31" s="21" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="22" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="B32" s="22" t="s">
         <v>15</v>
       </c>
       <c r="C32" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D32" s="22" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="22" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="B33" s="22" t="s">
         <v>16</v>
       </c>
       <c r="C33" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D33" s="22" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="22" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="B34" s="22" t="s">
         <v>17</v>
       </c>
       <c r="C34" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D34" s="22" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="22" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="B35" s="22" t="s">
         <v>18</v>
       </c>
       <c r="C35" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D35" s="22" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="22" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="B36" s="22" t="s">
         <v>19</v>
       </c>
       <c r="C36" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D36" s="22" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="B37" s="22" t="s">
         <v>20</v>
       </c>
       <c r="C37" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D37" s="22" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="21" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="B38" s="21" t="s">
         <v>21</v>
       </c>
       <c r="C38" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D38" s="21" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="22" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B39" s="22" t="s">
         <v>22</v>
       </c>
       <c r="C39" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D39" s="22" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="21" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="B40" s="21" t="s">
-        <v>197</v>
+        <v>23</v>
       </c>
       <c r="C40" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D40" s="21" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="21" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B41" s="21" t="s">
-        <v>200</v>
+        <v>24</v>
       </c>
       <c r="C41" s="21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D41" s="21" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="22" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B42" s="22" t="s">
         <v>25</v>
       </c>
       <c r="C42" s="22" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D42" s="22" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="19" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="B45" s="23" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="C45" s="23"/>
       <c r="D45" s="23"/>
     </row>
     <row r="46" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="18" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="B46" s="24" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C46" s="24" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="D46" s="24" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="18" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="B47" s="25" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="C47" s="25" t="n">
         <v>204</v>
       </c>
       <c r="D47" s="25" t="s">
-        <v>212</v>
+        <v>205</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="18" t="s">
-        <v>213</v>
+        <v>206</v>
       </c>
       <c r="B48" s="25" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="C48" s="25" t="n">
         <v>207</v>
       </c>
       <c r="D48" s="25" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="18" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="B49" s="25" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C49" s="25" t="n">
         <v>27</v>
       </c>
       <c r="D49" s="25" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B50" s="25" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="C50" s="25" t="n">
         <v>28</v>
       </c>
       <c r="D50" s="25" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B51" s="25" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="C51" s="25" t="n">
         <v>201</v>
       </c>
       <c r="D51" s="25" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B52" s="25" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="C52" s="25" t="n">
         <v>202</v>
       </c>
       <c r="D52" s="25" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>